<commit_message>
Carta de liberación y registro de proyecto
</commit_message>
<xml_diff>
--- a/Registro_proyecto_estadias_Yismael_Diaz.xlsx
+++ b/Registro_proyecto_estadias_Yismael_Diaz.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\estadias\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\diazy13\Documents\Estadias\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14EAF109-3D4D-4131-A9CB-A974A6A3A674}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BA5326C-5142-4B49-AE60-347EB33E49AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Asignación de Proyecto" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Asignación de Proyecto'!$A$2:$L$37</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'Formato de Asesorías'!$A$2:$L$33</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Formato de Asesorías'!$A$2:$L$43</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -34,15 +34,12 @@
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="121">
   <si>
     <t>Registro del proyecto de estadías</t>
   </si>
@@ -272,24 +269,12 @@
     <t>Correo electrónico (CE)</t>
   </si>
   <si>
-    <t>Asesoría inicial para informar el sistema de trabajo</t>
-  </si>
-  <si>
-    <t>Revisión del capitulo 1</t>
-  </si>
-  <si>
     <t>Se establecen fechas para proximas asesorias.</t>
   </si>
   <si>
     <t>Se realizan correcciones en capitulo 1.</t>
   </si>
   <si>
-    <t>Revisión de capitulo 2 y del registro de proyecto de estadias.</t>
-  </si>
-  <si>
-    <t>Retroalimentación de cap. 1 y corrección en capitulo 2 y registro de proyecto</t>
-  </si>
-  <si>
     <t>V</t>
   </si>
   <si>
@@ -324,6 +309,120 @@
   </si>
   <si>
     <t xml:space="preserve">4. Establecer un mecanismo de trazabilidad y generación de reportes auditables, asegurando la integridad de la información para fines de control de calidad. </t>
+  </si>
+  <si>
+    <t>PEEM</t>
+  </si>
+  <si>
+    <t>Se explicó detalladamente el proceso que debía digitalizarse, así como los puntos clave a considerar para su desarrollo.</t>
+  </si>
+  <si>
+    <t>Se definieron los plazos para la ejecución del proyecto y la documentación necesaria por parte de ambos involucrados.</t>
+  </si>
+  <si>
+    <t>Retroalimentación de cap. 1 y corrección en capitulo 2 y registro de proyecto.</t>
+  </si>
+  <si>
+    <t>Revisión de capitulo 2 y del registro de proyecto de estadias por la asesora universitaria.</t>
+  </si>
+  <si>
+    <t>Reunión grupal con la asesora universitaria para información del cierre de estadías.</t>
+  </si>
+  <si>
+    <t>Sesión complementaria con los involucrados internos de la empresa.</t>
+  </si>
+  <si>
+    <t>Primer acercamiento con el asesor empresarial.</t>
+  </si>
+  <si>
+    <t>Asesoría universitaria inicial para informar el sistema de trabajo.</t>
+  </si>
+  <si>
+    <t>Se informó el proceso y fechas próximas para el fin de estadias.</t>
+  </si>
+  <si>
+    <t>PEUTEZ</t>
+  </si>
+  <si>
+    <t>Revisión del capitulo 3.1 Inicio y 3.2 Planeación por la asesora universitaria.</t>
+  </si>
+  <si>
+    <t>Correcciones de los esquemas y diagramas usados.</t>
+  </si>
+  <si>
+    <t>Debido a cambios grandes necesarios en el reporte se tuvo la necesidad de realizar una segunda reunión el mismo día para finalizar la revisión.</t>
+  </si>
+  <si>
+    <t>Se revisó el contenido adicional a los capitulos para finalizar el reporte.</t>
+  </si>
+  <si>
+    <t>Revisión con el asesor universitario del inicio de sesión y página principal.</t>
+  </si>
+  <si>
+    <t>Revisión con el asesor universitario de los diseños de interfaz.</t>
+  </si>
+  <si>
+    <t>Revisión del capitulo 1 por la asesora universitaria.</t>
+  </si>
+  <si>
+    <t>Revisión del capitulo 4, el resumen y los indices.</t>
+  </si>
+  <si>
+    <t>Revisión completa del capitulo 3.</t>
+  </si>
+  <si>
+    <t>Revisión del capitulo 3.3 Ejecución.</t>
+  </si>
+  <si>
+    <t>Se analizaron distintas formas para el manejo del flujo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Se reorganizó la estructura de la ejecución y añadieron los puntos 3.3.5 Seguridad y 3.3.7 Despliegue.</t>
+  </si>
+  <si>
+    <t>Se dio visto bueno y se continuó con el desarrollo de los módulos.</t>
+  </si>
+  <si>
+    <t>Revisión con el equipo de manufactura para el módulo de creación de lotes.</t>
+  </si>
+  <si>
+    <t>Se aceptó el flujo para la creación del lote</t>
+  </si>
+  <si>
+    <t>Revisión de la aprobación del lote y generación de etiquetas.</t>
+  </si>
+  <si>
+    <t>Se aceptó la estructura de las etiquetas y las funciones de aprobación y rechazo del lote.</t>
+  </si>
+  <si>
+    <t>Revisión del módulo de registro de cajas y vinculación de muestras.</t>
+  </si>
+  <si>
+    <t>Se probó junto con el equipo del área de calidad la función para registro de cajas y vinculación a las muestras retenidas.</t>
+  </si>
+  <si>
+    <t>Se validó la manera de registrar y visualizar los estantes de los almaneces.</t>
+  </si>
+  <si>
+    <t>Revisión de la generación de almacenes y sus códigos QR.</t>
+  </si>
+  <si>
+    <t>Revisión de la vinculación de cajas con los estantes de almacén por código QR.</t>
+  </si>
+  <si>
+    <t>Se verificó el flujo completo de la aplicación para detectar posibles errores con los distintos códigos QR generados.</t>
+  </si>
+  <si>
+    <t>Revisión de inspección anual de lote.</t>
+  </si>
+  <si>
+    <t>Con el equipo del área de calidad se validó el fin del flujo del sistema pasando por los módulos planteados al inicio del proyecto.</t>
+  </si>
+  <si>
+    <t>Reunión con la directora del área de calidad.</t>
+  </si>
+  <si>
+    <t>El proyecto fue revisado por la directora de calidad de Vantive México mostrando su aprobación y grandes espectativas para la mejora continua del proceso.</t>
   </si>
 </sst>
 </file>
@@ -415,7 +514,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="55">
+  <borders count="64">
     <border>
       <left/>
       <right/>
@@ -718,50 +817,7 @@
       <left style="medium">
         <color theme="1" tint="0.499984740745262"/>
       </left>
-      <right style="medium">
-        <color theme="1" tint="0.499984740745262"/>
-      </right>
-      <top/>
-      <bottom style="medium">
-        <color theme="1" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color theme="1" tint="0.499984740745262"/>
-      </left>
       <right style="thin">
-        <color theme="1" tint="0.499984740745262"/>
-      </right>
-      <top style="medium">
-        <color theme="1" tint="0.499984740745262"/>
-      </top>
-      <bottom style="thin">
-        <color theme="1" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="1" tint="0.499984740745262"/>
-      </left>
-      <right style="thin">
-        <color theme="1" tint="0.499984740745262"/>
-      </right>
-      <top style="medium">
-        <color theme="1" tint="0.499984740745262"/>
-      </top>
-      <bottom style="thin">
-        <color theme="1" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="1" tint="0.499984740745262"/>
-      </left>
-      <right style="medium">
         <color theme="1" tint="0.499984740745262"/>
       </right>
       <top style="medium">
@@ -1033,12 +1089,166 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color theme="1" tint="0.499984740745262"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color theme="1" tint="0.499984740745262"/>
+      </top>
+      <bottom style="thin">
+        <color theme="1" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="1" tint="0.499984740745262"/>
+      </right>
+      <top style="thin">
+        <color theme="1" tint="0.499984740745262"/>
+      </top>
+      <bottom style="thin">
+        <color theme="1" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color theme="1" tint="0.499984740745262"/>
+      </left>
+      <right style="medium">
+        <color theme="1" tint="0.499984740745262"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color theme="1" tint="0.499984740745262"/>
+      </left>
+      <right style="thin">
+        <color theme="1" tint="0.499984740745262"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color theme="1" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="1" tint="0.499984740745262"/>
+      </left>
+      <right style="thin">
+        <color theme="1" tint="0.499984740745262"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color theme="1" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="1" tint="0.499984740745262"/>
+      </left>
+      <right style="medium">
+        <color theme="1" tint="0.499984740745262"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color theme="1" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color theme="1" tint="0.499984740745262"/>
+      </top>
+      <bottom style="thin">
+        <color theme="1" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color theme="1" tint="0.499984740745262"/>
+      </top>
+      <bottom style="thin">
+        <color theme="1" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="194">
+  <cellXfs count="220">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyProtection="1">
       <protection locked="0"/>
@@ -1122,6 +1332,10 @@
     <xf numFmtId="49" fontId="2" fillId="0" borderId="25" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="14" fontId="5" fillId="0" borderId="28" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="14" fontId="5" fillId="0" borderId="29" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
@@ -1130,34 +1344,26 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="14" fontId="5" fillId="0" borderId="35" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="40" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="37" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="41" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="38" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="43" xfId="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="45" xfId="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="46" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="40" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="42" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="43" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1183,6 +1389,313 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="justify" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="justify" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="justify" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="justify" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="justify" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="justify" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="justify" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="5" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="5" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="5" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="5" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="justify" vertical="justify" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="justify" vertical="justify" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="justify" vertical="justify" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1213,24 +1726,7 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="14" fontId="5" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1239,7 +1735,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1251,16 +1747,16 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="justify" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1270,426 +1766,245 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="30" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="33" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="33" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="31" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="34" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="5" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="5" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="5" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="justify" vertical="justify" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="justify" vertical="justify" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="justify" vertical="justify" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="54" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="justify" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="justify" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="justify" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="justify" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="justify" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="justify" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="27" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="28" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="25" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="25" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="26" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="27" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="25" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="36" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="37" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="39" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="41" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="42" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="30" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="30" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="52" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="53" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="52" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="55" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="33" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="55" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="34" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="55" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="5" fillId="0" borderId="56" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="30" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="30" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="57" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="31" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="58" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="33" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="59" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="61" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="59" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="60" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="61" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="5" fillId="0" borderId="54" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="57" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="52" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="53" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="52" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="54" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="54" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="57" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="19" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="33" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="36" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="39" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="40" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="42" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="44" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="45" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="62" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="63" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="28" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="25" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="25" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="26" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="27" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="28" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="25" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="36" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="37" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <protection locked="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1829,9 +2144,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
-      <xdr:colOff>1608736</xdr:colOff>
+      <xdr:colOff>1620166</xdr:colOff>
       <xdr:row>4</xdr:row>
-      <xdr:rowOff>65932</xdr:rowOff>
+      <xdr:rowOff>60217</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1874,13 +2189,13 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>25400</xdr:colOff>
-      <xdr:row>30</xdr:row>
+      <xdr:row>40</xdr:row>
       <xdr:rowOff>63500</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
       <xdr:colOff>1692275</xdr:colOff>
-      <xdr:row>33</xdr:row>
+      <xdr:row>43</xdr:row>
       <xdr:rowOff>1811</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -2295,58 +2610,58 @@
   <sheetData>
     <row r="1" spans="1:15" ht="3.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="1:15" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="124" t="s">
+      <c r="A2" s="92" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="125"/>
-      <c r="C2" s="125"/>
-      <c r="D2" s="125"/>
-      <c r="E2" s="125"/>
-      <c r="F2" s="125"/>
-      <c r="G2" s="125"/>
-      <c r="H2" s="125"/>
-      <c r="I2" s="125"/>
-      <c r="J2" s="125"/>
-      <c r="K2" s="104"/>
-      <c r="L2" s="105"/>
+      <c r="B2" s="93"/>
+      <c r="C2" s="93"/>
+      <c r="D2" s="93"/>
+      <c r="E2" s="93"/>
+      <c r="F2" s="93"/>
+      <c r="G2" s="93"/>
+      <c r="H2" s="93"/>
+      <c r="I2" s="93"/>
+      <c r="J2" s="93"/>
+      <c r="K2" s="72"/>
+      <c r="L2" s="73"/>
       <c r="N2" s="6" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:15" ht="23.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="126" t="s">
+      <c r="A3" s="94" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="127"/>
-      <c r="C3" s="127"/>
-      <c r="D3" s="127"/>
-      <c r="E3" s="127"/>
-      <c r="F3" s="127"/>
-      <c r="G3" s="127"/>
-      <c r="H3" s="127"/>
-      <c r="I3" s="127"/>
-      <c r="J3" s="127"/>
-      <c r="K3" s="106"/>
-      <c r="L3" s="107"/>
+      <c r="B3" s="95"/>
+      <c r="C3" s="95"/>
+      <c r="D3" s="95"/>
+      <c r="E3" s="95"/>
+      <c r="F3" s="95"/>
+      <c r="G3" s="95"/>
+      <c r="H3" s="95"/>
+      <c r="I3" s="95"/>
+      <c r="J3" s="95"/>
+      <c r="K3" s="74"/>
+      <c r="L3" s="75"/>
       <c r="N3" s="6" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:15" ht="23.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="128" t="s">
+      <c r="A4" s="96" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="129"/>
-      <c r="C4" s="129"/>
-      <c r="D4" s="129"/>
-      <c r="E4" s="129"/>
-      <c r="F4" s="129"/>
-      <c r="G4" s="129"/>
-      <c r="H4" s="129"/>
-      <c r="I4" s="129"/>
-      <c r="J4" s="129"/>
-      <c r="K4" s="108"/>
-      <c r="L4" s="109"/>
+      <c r="B4" s="97"/>
+      <c r="C4" s="97"/>
+      <c r="D4" s="97"/>
+      <c r="E4" s="97"/>
+      <c r="F4" s="97"/>
+      <c r="G4" s="97"/>
+      <c r="H4" s="97"/>
+      <c r="I4" s="97"/>
+      <c r="J4" s="97"/>
+      <c r="K4" s="76"/>
+      <c r="L4" s="77"/>
       <c r="N4" s="6" t="s">
         <v>5</v>
       </c>
@@ -2355,183 +2670,183 @@
       <c r="A5" s="29" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="130" t="s">
+      <c r="B5" s="98" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="130"/>
-      <c r="D5" s="130"/>
-      <c r="E5" s="130"/>
-      <c r="F5" s="130"/>
-      <c r="G5" s="130"/>
-      <c r="H5" s="130"/>
-      <c r="I5" s="130"/>
-      <c r="J5" s="130"/>
-      <c r="K5" s="130"/>
-      <c r="L5" s="131"/>
+      <c r="C5" s="98"/>
+      <c r="D5" s="98"/>
+      <c r="E5" s="98"/>
+      <c r="F5" s="98"/>
+      <c r="G5" s="98"/>
+      <c r="H5" s="98"/>
+      <c r="I5" s="98"/>
+      <c r="J5" s="98"/>
+      <c r="K5" s="98"/>
+      <c r="L5" s="99"/>
       <c r="N5" s="6" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="6" spans="1:15" s="6" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="43" t="s">
+      <c r="A6" s="42" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="81">
+      <c r="B6" s="105">
         <v>26</v>
       </c>
-      <c r="C6" s="81"/>
-      <c r="D6" s="81"/>
-      <c r="E6" s="81"/>
-      <c r="F6" s="81"/>
-      <c r="G6" s="81"/>
-      <c r="H6" s="40"/>
-      <c r="I6" s="80" t="s">
+      <c r="C6" s="105"/>
+      <c r="D6" s="105"/>
+      <c r="E6" s="105"/>
+      <c r="F6" s="105"/>
+      <c r="G6" s="105"/>
+      <c r="H6" s="39"/>
+      <c r="I6" s="130" t="s">
         <v>10</v>
       </c>
-      <c r="J6" s="80"/>
-      <c r="K6" s="78" t="s">
+      <c r="J6" s="130"/>
+      <c r="K6" s="106" t="s">
         <v>11</v>
       </c>
-      <c r="L6" s="79"/>
-      <c r="N6" s="38" t="s">
+      <c r="L6" s="107"/>
+      <c r="N6" s="13" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="7" spans="1:15" s="6" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="43" t="s">
+      <c r="A7" s="42" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="81" t="s">
+      <c r="B7" s="105" t="s">
         <v>14</v>
       </c>
-      <c r="C7" s="81"/>
-      <c r="D7" s="81"/>
-      <c r="E7" s="81"/>
-      <c r="F7" s="81"/>
-      <c r="G7" s="81"/>
-      <c r="H7" s="40"/>
-      <c r="I7" s="80" t="s">
+      <c r="C7" s="105"/>
+      <c r="D7" s="105"/>
+      <c r="E7" s="105"/>
+      <c r="F7" s="105"/>
+      <c r="G7" s="105"/>
+      <c r="H7" s="39"/>
+      <c r="I7" s="130" t="s">
         <v>15</v>
       </c>
-      <c r="J7" s="80"/>
-      <c r="K7" s="78" t="s">
+      <c r="J7" s="130"/>
+      <c r="K7" s="106" t="s">
         <v>16</v>
       </c>
-      <c r="L7" s="79"/>
-      <c r="N7" s="38" t="s">
+      <c r="L7" s="107"/>
+      <c r="N7" s="13" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="8" spans="1:15" s="6" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="43" t="s">
+      <c r="A8" s="42" t="s">
         <v>18</v>
       </c>
-      <c r="B8" s="78" t="s">
+      <c r="B8" s="106" t="s">
         <v>19</v>
       </c>
-      <c r="C8" s="78"/>
-      <c r="D8" s="78"/>
-      <c r="E8" s="78"/>
-      <c r="F8" s="78"/>
-      <c r="G8" s="78"/>
-      <c r="H8" s="78"/>
-      <c r="I8" s="80" t="s">
+      <c r="C8" s="106"/>
+      <c r="D8" s="106"/>
+      <c r="E8" s="106"/>
+      <c r="F8" s="106"/>
+      <c r="G8" s="106"/>
+      <c r="H8" s="106"/>
+      <c r="I8" s="130" t="s">
         <v>20</v>
       </c>
-      <c r="J8" s="80"/>
-      <c r="K8" s="81" t="s">
+      <c r="J8" s="130"/>
+      <c r="K8" s="105" t="s">
         <v>21</v>
       </c>
-      <c r="L8" s="82"/>
-      <c r="N8" s="38" t="s">
+      <c r="L8" s="131"/>
+      <c r="N8" s="13" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="9" spans="1:15" s="6" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="43" t="s">
+      <c r="A9" s="42" t="s">
         <v>23</v>
       </c>
-      <c r="B9" s="81" t="s">
+      <c r="B9" s="105" t="s">
         <v>24</v>
       </c>
-      <c r="C9" s="81"/>
-      <c r="D9" s="81"/>
-      <c r="E9" s="81"/>
-      <c r="F9" s="81"/>
-      <c r="G9" s="81"/>
-      <c r="H9" s="81"/>
-      <c r="I9" s="81"/>
-      <c r="J9" s="81"/>
-      <c r="K9" s="81"/>
-      <c r="L9" s="82"/>
-      <c r="N9" s="38" t="s">
+      <c r="C9" s="105"/>
+      <c r="D9" s="105"/>
+      <c r="E9" s="105"/>
+      <c r="F9" s="105"/>
+      <c r="G9" s="105"/>
+      <c r="H9" s="105"/>
+      <c r="I9" s="105"/>
+      <c r="J9" s="105"/>
+      <c r="K9" s="105"/>
+      <c r="L9" s="131"/>
+      <c r="N9" s="13" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="10" spans="1:15" s="6" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="43" t="s">
+      <c r="A10" s="42" t="s">
         <v>3</v>
       </c>
-      <c r="B10" s="78" t="s">
+      <c r="B10" s="106" t="s">
         <v>26</v>
       </c>
-      <c r="C10" s="78"/>
-      <c r="D10" s="78"/>
-      <c r="E10" s="78"/>
-      <c r="F10" s="78"/>
-      <c r="G10" s="78"/>
-      <c r="H10" s="78"/>
-      <c r="I10" s="78"/>
-      <c r="J10" s="78"/>
-      <c r="K10" s="78"/>
-      <c r="L10" s="79"/>
-      <c r="N10" s="38" t="s">
+      <c r="C10" s="106"/>
+      <c r="D10" s="106"/>
+      <c r="E10" s="106"/>
+      <c r="F10" s="106"/>
+      <c r="G10" s="106"/>
+      <c r="H10" s="106"/>
+      <c r="I10" s="106"/>
+      <c r="J10" s="106"/>
+      <c r="K10" s="106"/>
+      <c r="L10" s="107"/>
+      <c r="N10" s="13" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="11" spans="1:15" s="6" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="43" t="s">
+      <c r="A11" s="42" t="s">
         <v>5</v>
       </c>
-      <c r="B11" s="78" t="s">
-        <v>76</v>
-      </c>
-      <c r="C11" s="78"/>
-      <c r="D11" s="78"/>
-      <c r="E11" s="78"/>
-      <c r="F11" s="78"/>
-      <c r="G11" s="78"/>
-      <c r="H11" s="78"/>
-      <c r="I11" s="78"/>
-      <c r="J11" s="78"/>
-      <c r="K11" s="78"/>
-      <c r="L11" s="79"/>
-      <c r="N11" s="38" t="s">
+      <c r="B11" s="106" t="s">
+        <v>72</v>
+      </c>
+      <c r="C11" s="106"/>
+      <c r="D11" s="106"/>
+      <c r="E11" s="106"/>
+      <c r="F11" s="106"/>
+      <c r="G11" s="106"/>
+      <c r="H11" s="106"/>
+      <c r="I11" s="106"/>
+      <c r="J11" s="106"/>
+      <c r="K11" s="106"/>
+      <c r="L11" s="107"/>
+      <c r="N11" s="13" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="12" spans="1:15" s="6" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="43" t="s">
+      <c r="A12" s="42" t="s">
         <v>29</v>
       </c>
-      <c r="B12" s="132">
+      <c r="B12" s="100">
         <v>46028</v>
       </c>
-      <c r="C12" s="132"/>
-      <c r="D12" s="132"/>
-      <c r="E12" s="132"/>
+      <c r="C12" s="100"/>
+      <c r="D12" s="100"/>
+      <c r="E12" s="100"/>
       <c r="F12" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="G12" s="133">
+      <c r="G12" s="101">
         <v>46128</v>
       </c>
-      <c r="H12" s="133"/>
-      <c r="I12" s="133"/>
-      <c r="J12" s="133"/>
-      <c r="K12" s="133"/>
-      <c r="L12" s="134"/>
-      <c r="N12" s="38" t="s">
+      <c r="H12" s="101"/>
+      <c r="I12" s="101"/>
+      <c r="J12" s="101"/>
+      <c r="K12" s="101"/>
+      <c r="L12" s="102"/>
+      <c r="N12" s="13" t="s">
         <v>31</v>
       </c>
     </row>
@@ -2539,13 +2854,13 @@
       <c r="A13" s="19" t="s">
         <v>32</v>
       </c>
-      <c r="B13" s="123" t="s">
+      <c r="B13" s="91" t="s">
         <v>25</v>
       </c>
-      <c r="C13" s="123"/>
-      <c r="D13" s="123"/>
-      <c r="E13" s="123"/>
-      <c r="F13" s="123"/>
+      <c r="C13" s="91"/>
+      <c r="D13" s="91"/>
+      <c r="E13" s="91"/>
+      <c r="F13" s="91"/>
       <c r="G13" s="14"/>
       <c r="H13" s="14"/>
       <c r="I13" s="14"/>
@@ -2554,435 +2869,451 @@
       <c r="L13" s="16"/>
     </row>
     <row r="14" spans="1:15" s="6" customFormat="1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="46" t="s">
+      <c r="A14" s="132" t="s">
         <v>33</v>
       </c>
-      <c r="B14" s="47"/>
-      <c r="C14" s="47"/>
-      <c r="D14" s="47"/>
-      <c r="E14" s="47"/>
-      <c r="F14" s="110" t="s">
+      <c r="B14" s="133"/>
+      <c r="C14" s="133"/>
+      <c r="D14" s="133"/>
+      <c r="E14" s="133"/>
+      <c r="F14" s="78" t="s">
         <v>34</v>
       </c>
-      <c r="G14" s="111"/>
-      <c r="H14" s="111"/>
-      <c r="I14" s="111"/>
-      <c r="J14" s="111"/>
-      <c r="K14" s="111"/>
-      <c r="L14" s="112"/>
+      <c r="G14" s="79"/>
+      <c r="H14" s="79"/>
+      <c r="I14" s="79"/>
+      <c r="J14" s="79"/>
+      <c r="K14" s="79"/>
+      <c r="L14" s="80"/>
       <c r="M14" s="9"/>
       <c r="O14" s="9"/>
     </row>
     <row r="15" spans="1:15" s="6" customFormat="1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="75" t="s">
+      <c r="A15" s="45" t="s">
         <v>35</v>
       </c>
-      <c r="B15" s="76"/>
-      <c r="C15" s="76"/>
-      <c r="D15" s="76"/>
-      <c r="E15" s="77"/>
-      <c r="F15" s="56" t="s">
-        <v>77</v>
-      </c>
-      <c r="G15" s="57"/>
-      <c r="H15" s="57"/>
-      <c r="I15" s="57"/>
-      <c r="J15" s="57"/>
-      <c r="K15" s="57"/>
-      <c r="L15" s="58"/>
+      <c r="B15" s="46"/>
+      <c r="C15" s="46"/>
+      <c r="D15" s="46"/>
+      <c r="E15" s="47"/>
+      <c r="F15" s="62" t="s">
+        <v>73</v>
+      </c>
+      <c r="G15" s="46"/>
+      <c r="H15" s="46"/>
+      <c r="I15" s="46"/>
+      <c r="J15" s="46"/>
+      <c r="K15" s="46"/>
+      <c r="L15" s="63"/>
       <c r="M15" s="9"/>
       <c r="O15" s="9"/>
     </row>
     <row r="16" spans="1:15" s="6" customFormat="1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="75"/>
-      <c r="B16" s="76"/>
-      <c r="C16" s="76"/>
-      <c r="D16" s="76"/>
-      <c r="E16" s="77"/>
-      <c r="F16" s="56" t="s">
-        <v>78</v>
-      </c>
-      <c r="G16" s="57"/>
-      <c r="H16" s="57"/>
-      <c r="I16" s="57"/>
-      <c r="J16" s="57"/>
-      <c r="K16" s="57"/>
-      <c r="L16" s="58"/>
+      <c r="A16" s="45"/>
+      <c r="B16" s="46"/>
+      <c r="C16" s="46"/>
+      <c r="D16" s="46"/>
+      <c r="E16" s="47"/>
+      <c r="F16" s="62" t="s">
+        <v>74</v>
+      </c>
+      <c r="G16" s="46"/>
+      <c r="H16" s="46"/>
+      <c r="I16" s="46"/>
+      <c r="J16" s="46"/>
+      <c r="K16" s="46"/>
+      <c r="L16" s="63"/>
       <c r="M16" s="9"/>
       <c r="O16" s="9"/>
     </row>
     <row r="17" spans="1:16" s="6" customFormat="1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="141"/>
-      <c r="B17" s="142"/>
-      <c r="C17" s="142"/>
-      <c r="D17" s="142"/>
-      <c r="E17" s="143"/>
-      <c r="F17" s="56" t="s">
-        <v>79</v>
-      </c>
-      <c r="G17" s="57"/>
-      <c r="H17" s="57"/>
-      <c r="I17" s="57"/>
-      <c r="J17" s="57"/>
-      <c r="K17" s="57"/>
-      <c r="L17" s="58"/>
+      <c r="A17" s="48"/>
+      <c r="B17" s="49"/>
+      <c r="C17" s="49"/>
+      <c r="D17" s="49"/>
+      <c r="E17" s="50"/>
+      <c r="F17" s="62" t="s">
+        <v>75</v>
+      </c>
+      <c r="G17" s="46"/>
+      <c r="H17" s="46"/>
+      <c r="I17" s="46"/>
+      <c r="J17" s="46"/>
+      <c r="K17" s="46"/>
+      <c r="L17" s="63"/>
       <c r="M17" s="9"/>
       <c r="O17" s="9"/>
     </row>
     <row r="18" spans="1:16" s="6" customFormat="1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="65" t="s">
+      <c r="A18" s="146" t="s">
         <v>36</v>
       </c>
-      <c r="B18" s="66"/>
-      <c r="C18" s="66"/>
-      <c r="D18" s="66"/>
-      <c r="E18" s="67"/>
-      <c r="F18" s="56" t="s">
-        <v>80</v>
-      </c>
-      <c r="G18" s="57"/>
-      <c r="H18" s="57"/>
-      <c r="I18" s="57"/>
-      <c r="J18" s="57"/>
-      <c r="K18" s="57"/>
-      <c r="L18" s="58"/>
+      <c r="B18" s="147"/>
+      <c r="C18" s="147"/>
+      <c r="D18" s="147"/>
+      <c r="E18" s="148"/>
+      <c r="F18" s="62" t="s">
+        <v>76</v>
+      </c>
+      <c r="G18" s="46"/>
+      <c r="H18" s="46"/>
+      <c r="I18" s="46"/>
+      <c r="J18" s="46"/>
+      <c r="K18" s="46"/>
+      <c r="L18" s="63"/>
       <c r="M18" s="9"/>
     </row>
     <row r="19" spans="1:16" s="6" customFormat="1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="149" t="s">
-        <v>81</v>
-      </c>
-      <c r="B19" s="150"/>
-      <c r="C19" s="150"/>
-      <c r="D19" s="150"/>
-      <c r="E19" s="151"/>
-      <c r="F19" s="45"/>
-      <c r="G19" s="38"/>
-      <c r="H19" s="38"/>
-      <c r="I19" s="38"/>
-      <c r="J19" s="38"/>
-      <c r="K19" s="38"/>
-      <c r="L19" s="39"/>
+      <c r="A19" s="56" t="s">
+        <v>77</v>
+      </c>
+      <c r="B19" s="57"/>
+      <c r="C19" s="57"/>
+      <c r="D19" s="57"/>
+      <c r="E19" s="58"/>
+      <c r="F19" s="44"/>
+      <c r="G19" s="13"/>
+      <c r="H19" s="13"/>
+      <c r="I19" s="13"/>
+      <c r="J19" s="13"/>
+      <c r="K19" s="13"/>
+      <c r="L19" s="38"/>
     </row>
     <row r="20" spans="1:16" s="6" customFormat="1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="149"/>
-      <c r="B20" s="150"/>
-      <c r="C20" s="150"/>
-      <c r="D20" s="150"/>
-      <c r="E20" s="151"/>
-      <c r="F20" s="45"/>
-      <c r="G20" s="38"/>
-      <c r="H20" s="38"/>
-      <c r="I20" s="38"/>
-      <c r="J20" s="38"/>
-      <c r="K20" s="38"/>
-      <c r="L20" s="39"/>
+      <c r="A20" s="56"/>
+      <c r="B20" s="57"/>
+      <c r="C20" s="57"/>
+      <c r="D20" s="57"/>
+      <c r="E20" s="58"/>
+      <c r="F20" s="44"/>
+      <c r="G20" s="13"/>
+      <c r="H20" s="13"/>
+      <c r="I20" s="13"/>
+      <c r="J20" s="13"/>
+      <c r="K20" s="13"/>
+      <c r="L20" s="38"/>
     </row>
     <row r="21" spans="1:16" s="6" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="152"/>
-      <c r="B21" s="153"/>
-      <c r="C21" s="153"/>
-      <c r="D21" s="153"/>
-      <c r="E21" s="154"/>
-      <c r="F21" s="135"/>
-      <c r="G21" s="135"/>
-      <c r="H21" s="135"/>
-      <c r="I21" s="135"/>
-      <c r="J21" s="135"/>
-      <c r="K21" s="135"/>
-      <c r="L21" s="136"/>
+      <c r="A21" s="59"/>
+      <c r="B21" s="60"/>
+      <c r="C21" s="60"/>
+      <c r="D21" s="60"/>
+      <c r="E21" s="61"/>
+      <c r="F21" s="103"/>
+      <c r="G21" s="103"/>
+      <c r="H21" s="103"/>
+      <c r="I21" s="103"/>
+      <c r="J21" s="103"/>
+      <c r="K21" s="103"/>
+      <c r="L21" s="104"/>
     </row>
     <row r="22" spans="1:16" s="6" customFormat="1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="62" t="s">
+      <c r="A22" s="143" t="s">
         <v>37</v>
       </c>
-      <c r="B22" s="63"/>
-      <c r="C22" s="63"/>
-      <c r="D22" s="63"/>
-      <c r="E22" s="64"/>
-      <c r="F22" s="113" t="s">
+      <c r="B22" s="144"/>
+      <c r="C22" s="144"/>
+      <c r="D22" s="144"/>
+      <c r="E22" s="145"/>
+      <c r="F22" s="81" t="s">
         <v>38</v>
       </c>
-      <c r="G22" s="114"/>
-      <c r="H22" s="114"/>
-      <c r="I22" s="114"/>
-      <c r="J22" s="115"/>
-      <c r="K22" s="119" t="s">
+      <c r="G22" s="82"/>
+      <c r="H22" s="82"/>
+      <c r="I22" s="82"/>
+      <c r="J22" s="83"/>
+      <c r="K22" s="87" t="s">
         <v>39</v>
       </c>
-      <c r="L22" s="120"/>
+      <c r="L22" s="88"/>
       <c r="N22" s="10"/>
       <c r="P22" s="7"/>
     </row>
     <row r="23" spans="1:16" s="6" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="146" t="s">
-        <v>83</v>
-      </c>
-      <c r="B23" s="147"/>
-      <c r="C23" s="147"/>
-      <c r="D23" s="147"/>
-      <c r="E23" s="148"/>
-      <c r="F23" s="116"/>
-      <c r="G23" s="117"/>
-      <c r="H23" s="117"/>
-      <c r="I23" s="117"/>
-      <c r="J23" s="118"/>
-      <c r="K23" s="121"/>
-      <c r="L23" s="122"/>
+      <c r="A23" s="53" t="s">
+        <v>79</v>
+      </c>
+      <c r="B23" s="54"/>
+      <c r="C23" s="54"/>
+      <c r="D23" s="54"/>
+      <c r="E23" s="55"/>
+      <c r="F23" s="84"/>
+      <c r="G23" s="85"/>
+      <c r="H23" s="85"/>
+      <c r="I23" s="85"/>
+      <c r="J23" s="86"/>
+      <c r="K23" s="89"/>
+      <c r="L23" s="90"/>
       <c r="P23" s="9"/>
     </row>
     <row r="24" spans="1:16" s="13" customFormat="1" ht="38.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="68" t="s">
-        <v>84</v>
-      </c>
-      <c r="B24" s="69"/>
-      <c r="C24" s="69"/>
-      <c r="D24" s="69"/>
-      <c r="E24" s="70"/>
-      <c r="F24" s="144" t="s">
+      <c r="A24" s="149" t="s">
+        <v>80</v>
+      </c>
+      <c r="B24" s="150"/>
+      <c r="C24" s="150"/>
+      <c r="D24" s="150"/>
+      <c r="E24" s="151"/>
+      <c r="F24" s="51" t="s">
         <v>40</v>
       </c>
-      <c r="G24" s="144"/>
-      <c r="H24" s="144"/>
-      <c r="I24" s="144"/>
-      <c r="J24" s="145"/>
-      <c r="K24" s="71">
+      <c r="G24" s="51"/>
+      <c r="H24" s="51"/>
+      <c r="I24" s="51"/>
+      <c r="J24" s="52"/>
+      <c r="K24" s="152">
         <v>46038</v>
       </c>
-      <c r="L24" s="55"/>
-      <c r="M24" s="38"/>
+      <c r="L24" s="68"/>
       <c r="N24" s="7"/>
-      <c r="O24" s="38"/>
       <c r="P24" s="7"/>
     </row>
     <row r="25" spans="1:16" s="13" customFormat="1" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="68" t="s">
-        <v>85</v>
-      </c>
-      <c r="B25" s="69"/>
-      <c r="C25" s="69"/>
-      <c r="D25" s="69"/>
-      <c r="E25" s="70"/>
-      <c r="F25" s="72" t="s">
+      <c r="A25" s="149" t="s">
+        <v>81</v>
+      </c>
+      <c r="B25" s="150"/>
+      <c r="C25" s="150"/>
+      <c r="D25" s="150"/>
+      <c r="E25" s="151"/>
+      <c r="F25" s="110" t="s">
         <v>41</v>
       </c>
-      <c r="G25" s="73"/>
-      <c r="H25" s="73"/>
-      <c r="I25" s="73"/>
-      <c r="J25" s="74"/>
-      <c r="K25" s="54">
+      <c r="G25" s="111"/>
+      <c r="H25" s="111"/>
+      <c r="I25" s="111"/>
+      <c r="J25" s="112"/>
+      <c r="K25" s="67">
         <v>46087</v>
       </c>
-      <c r="L25" s="55"/>
-      <c r="M25" s="38"/>
+      <c r="L25" s="68"/>
       <c r="N25" s="7"/>
-      <c r="O25" s="38"/>
       <c r="P25" s="7"/>
     </row>
     <row r="26" spans="1:16" s="13" customFormat="1" ht="46.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="68" t="s">
-        <v>86</v>
-      </c>
-      <c r="B26" s="69"/>
-      <c r="C26" s="69"/>
-      <c r="D26" s="69"/>
-      <c r="E26" s="70"/>
-      <c r="F26" s="72" t="s">
+      <c r="A26" s="149" t="s">
+        <v>82</v>
+      </c>
+      <c r="B26" s="150"/>
+      <c r="C26" s="150"/>
+      <c r="D26" s="150"/>
+      <c r="E26" s="151"/>
+      <c r="F26" s="110" t="s">
         <v>42</v>
       </c>
-      <c r="G26" s="73"/>
-      <c r="H26" s="73"/>
-      <c r="I26" s="73"/>
-      <c r="J26" s="74"/>
-      <c r="K26" s="54">
+      <c r="G26" s="111"/>
+      <c r="H26" s="111"/>
+      <c r="I26" s="111"/>
+      <c r="J26" s="112"/>
+      <c r="K26" s="67">
         <v>46108</v>
       </c>
-      <c r="L26" s="55"/>
-      <c r="M26" s="38"/>
+      <c r="L26" s="68"/>
       <c r="N26" s="7"/>
-      <c r="O26" s="38"/>
       <c r="P26" s="7"/>
     </row>
     <row r="27" spans="1:16" s="13" customFormat="1" ht="15" x14ac:dyDescent="0.25">
-      <c r="A27" s="96"/>
-      <c r="B27" s="97"/>
-      <c r="C27" s="97"/>
-      <c r="D27" s="97"/>
-      <c r="E27" s="98"/>
-      <c r="F27" s="72" t="s">
+      <c r="A27" s="124"/>
+      <c r="B27" s="125"/>
+      <c r="C27" s="125"/>
+      <c r="D27" s="125"/>
+      <c r="E27" s="126"/>
+      <c r="F27" s="110" t="s">
         <v>43</v>
       </c>
-      <c r="G27" s="73"/>
-      <c r="H27" s="73"/>
-      <c r="I27" s="73"/>
-      <c r="J27" s="74"/>
-      <c r="K27" s="54">
+      <c r="G27" s="111"/>
+      <c r="H27" s="111"/>
+      <c r="I27" s="111"/>
+      <c r="J27" s="112"/>
+      <c r="K27" s="67">
         <v>46122</v>
       </c>
-      <c r="L27" s="91"/>
-      <c r="M27" s="38"/>
-      <c r="N27" s="38"/>
-      <c r="O27" s="38"/>
-      <c r="P27" s="38"/>
+      <c r="L27" s="119"/>
     </row>
     <row r="28" spans="1:16" s="6" customFormat="1" ht="29.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="59" t="s">
+      <c r="A28" s="140" t="s">
         <v>44</v>
       </c>
-      <c r="B28" s="60"/>
-      <c r="C28" s="60"/>
-      <c r="D28" s="60"/>
-      <c r="E28" s="61"/>
-      <c r="F28" s="85" t="s">
+      <c r="B28" s="141"/>
+      <c r="C28" s="141"/>
+      <c r="D28" s="141"/>
+      <c r="E28" s="142"/>
+      <c r="F28" s="113" t="s">
         <v>45</v>
       </c>
-      <c r="G28" s="86"/>
-      <c r="H28" s="86"/>
-      <c r="I28" s="86"/>
-      <c r="J28" s="87"/>
-      <c r="K28" s="92">
+      <c r="G28" s="114"/>
+      <c r="H28" s="114"/>
+      <c r="I28" s="114"/>
+      <c r="J28" s="115"/>
+      <c r="K28" s="120">
         <v>46128</v>
       </c>
-      <c r="L28" s="93"/>
+      <c r="L28" s="121"/>
     </row>
     <row r="29" spans="1:16" s="6" customFormat="1" ht="63.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="99" t="s">
-        <v>82</v>
-      </c>
-      <c r="B29" s="100"/>
-      <c r="C29" s="100"/>
-      <c r="D29" s="100"/>
-      <c r="E29" s="101"/>
-      <c r="F29" s="88"/>
-      <c r="G29" s="89"/>
-      <c r="H29" s="89"/>
-      <c r="I29" s="89"/>
-      <c r="J29" s="90"/>
-      <c r="K29" s="54"/>
-      <c r="L29" s="55"/>
+      <c r="A29" s="127" t="s">
+        <v>78</v>
+      </c>
+      <c r="B29" s="128"/>
+      <c r="C29" s="128"/>
+      <c r="D29" s="128"/>
+      <c r="E29" s="129"/>
+      <c r="F29" s="116"/>
+      <c r="G29" s="117"/>
+      <c r="H29" s="117"/>
+      <c r="I29" s="117"/>
+      <c r="J29" s="118"/>
+      <c r="K29" s="67"/>
+      <c r="L29" s="68"/>
     </row>
     <row r="30" spans="1:16" s="6" customFormat="1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="48"/>
-      <c r="B30" s="49"/>
-      <c r="C30" s="49"/>
-      <c r="D30" s="49"/>
-      <c r="E30" s="50"/>
-      <c r="F30" s="88"/>
-      <c r="G30" s="89"/>
-      <c r="H30" s="89"/>
-      <c r="I30" s="89"/>
-      <c r="J30" s="90"/>
-      <c r="K30" s="54"/>
-      <c r="L30" s="55"/>
+      <c r="A30" s="134"/>
+      <c r="B30" s="135"/>
+      <c r="C30" s="135"/>
+      <c r="D30" s="135"/>
+      <c r="E30" s="136"/>
+      <c r="F30" s="116"/>
+      <c r="G30" s="117"/>
+      <c r="H30" s="117"/>
+      <c r="I30" s="117"/>
+      <c r="J30" s="118"/>
+      <c r="K30" s="67"/>
+      <c r="L30" s="68"/>
     </row>
     <row r="31" spans="1:16" s="6" customFormat="1" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="51"/>
-      <c r="B31" s="52"/>
-      <c r="C31" s="52"/>
-      <c r="D31" s="52"/>
-      <c r="E31" s="53"/>
-      <c r="F31" s="139"/>
-      <c r="G31" s="139"/>
-      <c r="H31" s="139"/>
-      <c r="I31" s="139"/>
-      <c r="J31" s="140"/>
-      <c r="K31" s="137"/>
-      <c r="L31" s="138"/>
+      <c r="A31" s="137"/>
+      <c r="B31" s="138"/>
+      <c r="C31" s="138"/>
+      <c r="D31" s="138"/>
+      <c r="E31" s="139"/>
+      <c r="F31" s="69"/>
+      <c r="G31" s="69"/>
+      <c r="H31" s="69"/>
+      <c r="I31" s="69"/>
+      <c r="J31" s="70"/>
+      <c r="K31" s="65"/>
+      <c r="L31" s="66"/>
     </row>
     <row r="32" spans="1:16" s="6" customFormat="1" ht="9.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="33" spans="1:12" s="6" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="103"/>
-      <c r="B33" s="103"/>
-      <c r="C33" s="103"/>
-      <c r="D33" s="103"/>
-      <c r="E33" s="41"/>
-      <c r="F33" s="103"/>
-      <c r="G33" s="103"/>
-      <c r="H33" s="103"/>
-      <c r="I33" s="103"/>
-      <c r="J33" s="103"/>
-      <c r="K33" s="103"/>
-      <c r="L33" s="103"/>
+      <c r="A33" s="71"/>
+      <c r="B33" s="71"/>
+      <c r="C33" s="71"/>
+      <c r="D33" s="71"/>
+      <c r="E33" s="40"/>
+      <c r="F33" s="71"/>
+      <c r="G33" s="71"/>
+      <c r="H33" s="71"/>
+      <c r="I33" s="71"/>
+      <c r="J33" s="71"/>
+      <c r="K33" s="71"/>
+      <c r="L33" s="71"/>
     </row>
     <row r="34" spans="1:12" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.25">
-      <c r="A34" s="102" t="str">
+      <c r="A34" s="64" t="str">
         <f>B10</f>
         <v>I. I. Julio César Torres Hernández</v>
       </c>
-      <c r="B34" s="102"/>
-      <c r="C34" s="102"/>
-      <c r="D34" s="102"/>
+      <c r="B34" s="64"/>
+      <c r="C34" s="64"/>
+      <c r="D34" s="64"/>
       <c r="E34" s="11"/>
-      <c r="F34" s="102" t="str">
+      <c r="F34" s="64" t="str">
         <f>B5</f>
         <v>Andrés Yismael Díaz Hernandéz</v>
       </c>
-      <c r="G34" s="102"/>
-      <c r="H34" s="102"/>
+      <c r="G34" s="64"/>
+      <c r="H34" s="64"/>
       <c r="I34" s="17"/>
-      <c r="J34" s="102" t="str">
+      <c r="J34" s="64" t="str">
         <f>B11</f>
         <v>M. C. Nélida Báron Pérez</v>
       </c>
-      <c r="K34" s="102"/>
-      <c r="L34" s="102"/>
+      <c r="K34" s="64"/>
+      <c r="L34" s="64"/>
     </row>
     <row r="35" spans="1:12" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.25">
-      <c r="A35" s="94" t="str">
+      <c r="A35" s="122" t="str">
         <f>UPPER(LEFT(A10, LEN(A10)-1))</f>
         <v>ASESOR EMPRESARIAL</v>
       </c>
-      <c r="B35" s="95"/>
-      <c r="C35" s="95"/>
-      <c r="D35" s="95"/>
+      <c r="B35" s="123"/>
+      <c r="C35" s="123"/>
+      <c r="D35" s="123"/>
       <c r="E35" s="5"/>
-      <c r="F35" s="94" t="s">
+      <c r="F35" s="122" t="s">
         <v>46</v>
       </c>
-      <c r="G35" s="94"/>
-      <c r="H35" s="94"/>
+      <c r="G35" s="122"/>
+      <c r="H35" s="122"/>
       <c r="I35" s="5"/>
-      <c r="J35" s="94" t="str">
+      <c r="J35" s="122" t="str">
         <f>UPPER(LEFT(A11, LEN(A11)-1))</f>
         <v>ASESORA UNIVERSITARIA</v>
       </c>
-      <c r="K35" s="94"/>
-      <c r="L35" s="94"/>
+      <c r="K35" s="122"/>
+      <c r="L35" s="122"/>
     </row>
     <row r="36" spans="1:12" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="83" t="s">
+      <c r="A36" s="108" t="s">
         <v>47</v>
       </c>
-      <c r="B36" s="84"/>
-      <c r="C36" s="84"/>
-      <c r="D36" s="84"/>
-      <c r="E36" s="84"/>
-      <c r="F36" s="84"/>
-      <c r="G36" s="84"/>
-      <c r="H36" s="84"/>
-      <c r="I36" s="84"/>
-      <c r="J36" s="84"/>
-      <c r="K36" s="84"/>
-      <c r="L36" s="84"/>
+      <c r="B36" s="109"/>
+      <c r="C36" s="109"/>
+      <c r="D36" s="109"/>
+      <c r="E36" s="109"/>
+      <c r="F36" s="109"/>
+      <c r="G36" s="109"/>
+      <c r="H36" s="109"/>
+      <c r="I36" s="109"/>
+      <c r="J36" s="109"/>
+      <c r="K36" s="109"/>
+      <c r="L36" s="109"/>
     </row>
     <row r="37" spans="1:12" ht="69" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <dataConsolidate/>
   <mergeCells count="70">
-    <mergeCell ref="A16:E16"/>
-    <mergeCell ref="A17:E17"/>
-    <mergeCell ref="F24:J24"/>
-    <mergeCell ref="A23:E23"/>
-    <mergeCell ref="A19:E21"/>
-    <mergeCell ref="F16:L16"/>
-    <mergeCell ref="F18:L18"/>
-    <mergeCell ref="F34:H34"/>
-    <mergeCell ref="K31:L31"/>
-    <mergeCell ref="A34:D34"/>
-    <mergeCell ref="K26:L26"/>
-    <mergeCell ref="F31:J31"/>
-    <mergeCell ref="F33:I33"/>
-    <mergeCell ref="J33:L33"/>
+    <mergeCell ref="A14:E14"/>
+    <mergeCell ref="A30:E30"/>
+    <mergeCell ref="A31:E31"/>
+    <mergeCell ref="K25:L25"/>
+    <mergeCell ref="F15:L15"/>
+    <mergeCell ref="F17:L17"/>
+    <mergeCell ref="A28:E28"/>
+    <mergeCell ref="A22:E22"/>
+    <mergeCell ref="A18:E18"/>
+    <mergeCell ref="A24:E24"/>
+    <mergeCell ref="A25:E25"/>
+    <mergeCell ref="A26:E26"/>
+    <mergeCell ref="K24:L24"/>
+    <mergeCell ref="F25:J25"/>
+    <mergeCell ref="F26:J26"/>
+    <mergeCell ref="A15:E15"/>
+    <mergeCell ref="B11:L11"/>
+    <mergeCell ref="I6:J6"/>
+    <mergeCell ref="I7:J7"/>
+    <mergeCell ref="I8:J8"/>
+    <mergeCell ref="B9:L9"/>
+    <mergeCell ref="K7:L7"/>
+    <mergeCell ref="K8:L8"/>
+    <mergeCell ref="B8:H8"/>
+    <mergeCell ref="A36:L36"/>
+    <mergeCell ref="K30:L30"/>
+    <mergeCell ref="F27:J27"/>
+    <mergeCell ref="F28:J28"/>
+    <mergeCell ref="F29:J29"/>
+    <mergeCell ref="F30:J30"/>
+    <mergeCell ref="K27:L27"/>
+    <mergeCell ref="K28:L28"/>
+    <mergeCell ref="K29:L29"/>
+    <mergeCell ref="A35:D35"/>
+    <mergeCell ref="J35:L35"/>
+    <mergeCell ref="F35:H35"/>
+    <mergeCell ref="A27:E27"/>
+    <mergeCell ref="A29:E29"/>
+    <mergeCell ref="J34:L34"/>
+    <mergeCell ref="A33:D33"/>
     <mergeCell ref="K2:L4"/>
     <mergeCell ref="F14:L14"/>
     <mergeCell ref="F22:J23"/>
@@ -2999,46 +3330,20 @@
     <mergeCell ref="B7:G7"/>
     <mergeCell ref="K6:L6"/>
     <mergeCell ref="B10:L10"/>
-    <mergeCell ref="A36:L36"/>
-    <mergeCell ref="K30:L30"/>
-    <mergeCell ref="F27:J27"/>
-    <mergeCell ref="F28:J28"/>
-    <mergeCell ref="F29:J29"/>
-    <mergeCell ref="F30:J30"/>
-    <mergeCell ref="K27:L27"/>
-    <mergeCell ref="K28:L28"/>
-    <mergeCell ref="K29:L29"/>
-    <mergeCell ref="A35:D35"/>
-    <mergeCell ref="J35:L35"/>
-    <mergeCell ref="F35:H35"/>
-    <mergeCell ref="A27:E27"/>
-    <mergeCell ref="A29:E29"/>
-    <mergeCell ref="J34:L34"/>
-    <mergeCell ref="A33:D33"/>
-    <mergeCell ref="B11:L11"/>
-    <mergeCell ref="I6:J6"/>
-    <mergeCell ref="I7:J7"/>
-    <mergeCell ref="I8:J8"/>
-    <mergeCell ref="B9:L9"/>
-    <mergeCell ref="K7:L7"/>
-    <mergeCell ref="K8:L8"/>
-    <mergeCell ref="B8:H8"/>
-    <mergeCell ref="A14:E14"/>
-    <mergeCell ref="A30:E30"/>
-    <mergeCell ref="A31:E31"/>
-    <mergeCell ref="K25:L25"/>
-    <mergeCell ref="F15:L15"/>
-    <mergeCell ref="F17:L17"/>
-    <mergeCell ref="A28:E28"/>
-    <mergeCell ref="A22:E22"/>
-    <mergeCell ref="A18:E18"/>
-    <mergeCell ref="A24:E24"/>
-    <mergeCell ref="A25:E25"/>
-    <mergeCell ref="A26:E26"/>
-    <mergeCell ref="K24:L24"/>
-    <mergeCell ref="F25:J25"/>
-    <mergeCell ref="F26:J26"/>
-    <mergeCell ref="A15:E15"/>
+    <mergeCell ref="F34:H34"/>
+    <mergeCell ref="K31:L31"/>
+    <mergeCell ref="A34:D34"/>
+    <mergeCell ref="K26:L26"/>
+    <mergeCell ref="F31:J31"/>
+    <mergeCell ref="F33:I33"/>
+    <mergeCell ref="J33:L33"/>
+    <mergeCell ref="A16:E16"/>
+    <mergeCell ref="A17:E17"/>
+    <mergeCell ref="F24:J24"/>
+    <mergeCell ref="A23:E23"/>
+    <mergeCell ref="A19:E21"/>
+    <mergeCell ref="F16:L16"/>
+    <mergeCell ref="F18:L18"/>
   </mergeCells>
   <phoneticPr fontId="0" type="noConversion"/>
   <dataValidations count="3">
@@ -3065,7 +3370,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:N33"/>
+  <dimension ref="A1:N43"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.44140625" style="1" customWidth="1"/>
@@ -3087,50 +3392,50 @@
   <sheetData>
     <row r="1" spans="1:14" ht="5.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="1:14" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="165" t="s">
+      <c r="A2" s="176" t="s">
         <v>48</v>
       </c>
-      <c r="B2" s="166"/>
-      <c r="C2" s="166"/>
-      <c r="D2" s="166"/>
-      <c r="E2" s="166"/>
-      <c r="F2" s="166"/>
-      <c r="G2" s="166"/>
-      <c r="H2" s="166"/>
-      <c r="I2" s="166"/>
-      <c r="J2" s="166"/>
+      <c r="B2" s="177"/>
+      <c r="C2" s="177"/>
+      <c r="D2" s="177"/>
+      <c r="E2" s="177"/>
+      <c r="F2" s="177"/>
+      <c r="G2" s="177"/>
+      <c r="H2" s="177"/>
+      <c r="I2" s="177"/>
+      <c r="J2" s="177"/>
       <c r="K2" s="33"/>
       <c r="L2" s="34"/>
     </row>
     <row r="3" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="167" t="s">
+      <c r="A3" s="178" t="s">
         <v>49</v>
       </c>
-      <c r="B3" s="168"/>
-      <c r="C3" s="168"/>
-      <c r="D3" s="168"/>
-      <c r="E3" s="168"/>
-      <c r="F3" s="168"/>
-      <c r="G3" s="168"/>
-      <c r="H3" s="168"/>
-      <c r="I3" s="168"/>
-      <c r="J3" s="168"/>
+      <c r="B3" s="179"/>
+      <c r="C3" s="179"/>
+      <c r="D3" s="179"/>
+      <c r="E3" s="179"/>
+      <c r="F3" s="179"/>
+      <c r="G3" s="179"/>
+      <c r="H3" s="179"/>
+      <c r="I3" s="179"/>
+      <c r="J3" s="179"/>
       <c r="K3" s="30"/>
       <c r="L3" s="35"/>
     </row>
     <row r="4" spans="1:14" ht="32.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="169" t="s">
+      <c r="A4" s="180" t="s">
         <v>50</v>
       </c>
-      <c r="B4" s="170"/>
-      <c r="C4" s="170"/>
-      <c r="D4" s="170"/>
-      <c r="E4" s="170"/>
-      <c r="F4" s="170"/>
-      <c r="G4" s="170"/>
-      <c r="H4" s="170"/>
-      <c r="I4" s="170"/>
-      <c r="J4" s="170"/>
+      <c r="B4" s="181"/>
+      <c r="C4" s="181"/>
+      <c r="D4" s="181"/>
+      <c r="E4" s="181"/>
+      <c r="F4" s="181"/>
+      <c r="G4" s="181"/>
+      <c r="H4" s="181"/>
+      <c r="I4" s="181"/>
+      <c r="J4" s="181"/>
       <c r="K4" s="36"/>
       <c r="L4" s="37"/>
     </row>
@@ -3139,19 +3444,19 @@
         <v>6</v>
       </c>
       <c r="B5" s="32"/>
-      <c r="C5" s="171" t="str">
+      <c r="C5" s="182" t="str">
         <f>'Asignación de Proyecto'!B5</f>
         <v>Andrés Yismael Díaz Hernandéz</v>
       </c>
-      <c r="D5" s="171"/>
-      <c r="E5" s="171"/>
-      <c r="F5" s="171"/>
-      <c r="G5" s="171"/>
-      <c r="H5" s="171"/>
-      <c r="I5" s="171"/>
-      <c r="J5" s="171"/>
-      <c r="K5" s="171"/>
-      <c r="L5" s="172"/>
+      <c r="D5" s="182"/>
+      <c r="E5" s="182"/>
+      <c r="F5" s="182"/>
+      <c r="G5" s="182"/>
+      <c r="H5" s="182"/>
+      <c r="I5" s="182"/>
+      <c r="J5" s="182"/>
+      <c r="K5" s="182"/>
+      <c r="L5" s="183"/>
       <c r="N5" s="2" t="s">
         <v>51</v>
       </c>
@@ -3160,8 +3465,8 @@
       <c r="A6" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="42"/>
-      <c r="C6" s="42">
+      <c r="B6" s="41"/>
+      <c r="C6" s="41">
         <f>'Asignación de Proyecto'!B6</f>
         <v>26</v>
       </c>
@@ -3174,21 +3479,21 @@
       <c r="J6" s="23" t="s">
         <v>52</v>
       </c>
-      <c r="K6" s="173" t="str">
+      <c r="K6" s="161" t="str">
         <f>'Asignación de Proyecto'!K6</f>
         <v>20243IGS003</v>
       </c>
-      <c r="L6" s="174"/>
+      <c r="L6" s="162"/>
       <c r="N6" s="2" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="7" spans="1:14" s="2" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="44" t="s">
+      <c r="A7" s="43" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="42"/>
-      <c r="C7" s="42" t="str">
+      <c r="B7" s="41"/>
+      <c r="C7" s="41" t="str">
         <f>'Asignación de Proyecto'!B7</f>
         <v>Ingeniería</v>
       </c>
@@ -3201,11 +3506,11 @@
       <c r="J7" s="23" t="s">
         <v>15</v>
       </c>
-      <c r="K7" s="173" t="str">
+      <c r="K7" s="161" t="str">
         <f>'Asignación de Proyecto'!K7</f>
         <v>11B</v>
       </c>
-      <c r="L7" s="174"/>
+      <c r="L7" s="162"/>
       <c r="N7" s="2" t="s">
         <v>54</v>
       </c>
@@ -3214,8 +3519,8 @@
       <c r="A8" s="20" t="s">
         <v>18</v>
       </c>
-      <c r="B8" s="42"/>
-      <c r="C8" s="42" t="str">
+      <c r="B8" s="41"/>
+      <c r="C8" s="41" t="str">
         <f xml:space="preserve"> 'Asignación de Proyecto'!B8</f>
         <v>Desarrollo y Gestión de Software</v>
       </c>
@@ -3228,434 +3533,741 @@
       <c r="J8" s="23" t="s">
         <v>55</v>
       </c>
-      <c r="K8" s="173" t="str">
+      <c r="K8" s="161" t="str">
         <f>'Asignación de Proyecto'!K8</f>
         <v>No aplica</v>
       </c>
-      <c r="L8" s="174"/>
+      <c r="L8" s="162"/>
     </row>
     <row r="9" spans="1:14" s="2" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="20" t="s">
         <v>23</v>
       </c>
       <c r="B9" s="24"/>
-      <c r="C9" s="175" t="str">
+      <c r="C9" s="163" t="str">
         <f>'Asignación de Proyecto'!B9</f>
         <v>Baxter S.A. de C.V.</v>
       </c>
-      <c r="D9" s="175"/>
-      <c r="E9" s="175"/>
-      <c r="F9" s="175"/>
-      <c r="G9" s="175"/>
-      <c r="H9" s="175"/>
-      <c r="I9" s="175"/>
-      <c r="J9" s="175"/>
-      <c r="K9" s="175"/>
-      <c r="L9" s="176"/>
+      <c r="D9" s="163"/>
+      <c r="E9" s="163"/>
+      <c r="F9" s="163"/>
+      <c r="G9" s="163"/>
+      <c r="H9" s="163"/>
+      <c r="I9" s="163"/>
+      <c r="J9" s="163"/>
+      <c r="K9" s="163"/>
+      <c r="L9" s="164"/>
     </row>
     <row r="10" spans="1:14" s="2" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="183" t="str">
+      <c r="A10" s="170" t="str">
         <f>'Asignación de Proyecto'!A10</f>
         <v>Asesor empresarial:</v>
       </c>
-      <c r="B10" s="184"/>
-      <c r="C10" s="173" t="str">
+      <c r="B10" s="171"/>
+      <c r="C10" s="161" t="str">
         <f>'Asignación de Proyecto'!B10</f>
         <v>I. I. Julio César Torres Hernández</v>
       </c>
-      <c r="D10" s="173"/>
-      <c r="E10" s="173"/>
-      <c r="F10" s="173"/>
-      <c r="G10" s="173"/>
-      <c r="H10" s="173"/>
-      <c r="I10" s="173"/>
-      <c r="J10" s="173"/>
-      <c r="K10" s="173"/>
-      <c r="L10" s="174"/>
+      <c r="D10" s="161"/>
+      <c r="E10" s="161"/>
+      <c r="F10" s="161"/>
+      <c r="G10" s="161"/>
+      <c r="H10" s="161"/>
+      <c r="I10" s="161"/>
+      <c r="J10" s="161"/>
+      <c r="K10" s="161"/>
+      <c r="L10" s="162"/>
     </row>
     <row r="11" spans="1:14" s="2" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="183" t="str">
+      <c r="A11" s="170" t="str">
         <f>'Asignación de Proyecto'!A11</f>
         <v>Asesora universitaria:</v>
       </c>
-      <c r="B11" s="184"/>
-      <c r="C11" s="173" t="str">
+      <c r="B11" s="171"/>
+      <c r="C11" s="161" t="str">
         <f>'Asignación de Proyecto'!B11</f>
         <v>M. C. Nélida Báron Pérez</v>
       </c>
-      <c r="D11" s="173"/>
-      <c r="E11" s="173"/>
-      <c r="F11" s="173"/>
-      <c r="G11" s="173"/>
-      <c r="H11" s="173"/>
-      <c r="I11" s="173"/>
-      <c r="J11" s="173"/>
-      <c r="K11" s="173"/>
-      <c r="L11" s="174"/>
+      <c r="D11" s="161"/>
+      <c r="E11" s="161"/>
+      <c r="F11" s="161"/>
+      <c r="G11" s="161"/>
+      <c r="H11" s="161"/>
+      <c r="I11" s="161"/>
+      <c r="J11" s="161"/>
+      <c r="K11" s="161"/>
+      <c r="L11" s="162"/>
     </row>
     <row r="12" spans="1:14" s="2" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="185" t="s">
+      <c r="A12" s="172" t="s">
         <v>33</v>
       </c>
-      <c r="B12" s="186"/>
-      <c r="C12" s="173" t="str">
+      <c r="B12" s="173"/>
+      <c r="C12" s="161" t="str">
         <f>'Asignación de Proyecto'!A15</f>
         <v>Monitoreo y Control de Muestras de Retención</v>
       </c>
-      <c r="D12" s="173"/>
-      <c r="E12" s="173"/>
-      <c r="F12" s="173"/>
-      <c r="G12" s="173"/>
-      <c r="H12" s="173"/>
-      <c r="I12" s="173"/>
-      <c r="J12" s="173"/>
-      <c r="K12" s="173"/>
-      <c r="L12" s="174"/>
+      <c r="D12" s="161"/>
+      <c r="E12" s="161"/>
+      <c r="F12" s="161"/>
+      <c r="G12" s="161"/>
+      <c r="H12" s="161"/>
+      <c r="I12" s="161"/>
+      <c r="J12" s="161"/>
+      <c r="K12" s="161"/>
+      <c r="L12" s="162"/>
     </row>
     <row r="13" spans="1:14" s="2" customFormat="1" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="187" t="s">
+      <c r="A13" s="174" t="s">
         <v>56</v>
       </c>
-      <c r="B13" s="188"/>
-      <c r="C13" s="178">
+      <c r="B13" s="175"/>
+      <c r="C13" s="166">
         <f>'Asignación de Proyecto'!B12</f>
         <v>46028</v>
       </c>
-      <c r="D13" s="178"/>
-      <c r="E13" s="178"/>
-      <c r="F13" s="178"/>
+      <c r="D13" s="166"/>
+      <c r="E13" s="166"/>
+      <c r="F13" s="166"/>
       <c r="G13" s="25" t="s">
         <v>57</v>
       </c>
-      <c r="H13" s="179">
+      <c r="H13" s="167">
         <f>'Asignación de Proyecto'!G12</f>
         <v>46128</v>
       </c>
-      <c r="I13" s="179"/>
-      <c r="J13" s="179"/>
-      <c r="K13" s="179"/>
-      <c r="L13" s="180"/>
+      <c r="I13" s="167"/>
+      <c r="J13" s="167"/>
+      <c r="K13" s="167"/>
+      <c r="L13" s="168"/>
     </row>
     <row r="14" spans="1:14" s="2" customFormat="1" ht="15" x14ac:dyDescent="0.25">
-      <c r="A14" s="155" t="s">
+      <c r="A14" s="165" t="s">
         <v>58</v>
       </c>
-      <c r="B14" s="181" t="s">
+      <c r="B14" s="169" t="s">
         <v>59</v>
       </c>
-      <c r="C14" s="181"/>
-      <c r="D14" s="181"/>
-      <c r="E14" s="181"/>
-      <c r="F14" s="155" t="s">
+      <c r="C14" s="169"/>
+      <c r="D14" s="169"/>
+      <c r="E14" s="169"/>
+      <c r="F14" s="165" t="s">
         <v>60</v>
       </c>
-      <c r="G14" s="155"/>
-      <c r="H14" s="181" t="s">
+      <c r="G14" s="165"/>
+      <c r="H14" s="169" t="s">
         <v>61</v>
       </c>
-      <c r="I14" s="181"/>
-      <c r="J14" s="181"/>
-      <c r="K14" s="155" t="s">
+      <c r="I14" s="169"/>
+      <c r="J14" s="169"/>
+      <c r="K14" s="165" t="s">
         <v>62</v>
       </c>
-      <c r="L14" s="155"/>
-    </row>
-    <row r="15" spans="1:14" s="2" customFormat="1" ht="15.6" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="156"/>
-      <c r="B15" s="182"/>
-      <c r="C15" s="182"/>
-      <c r="D15" s="182"/>
-      <c r="E15" s="182"/>
-      <c r="F15" s="177"/>
-      <c r="G15" s="177"/>
-      <c r="H15" s="182"/>
-      <c r="I15" s="182"/>
-      <c r="J15" s="182"/>
-      <c r="K15" s="177"/>
-      <c r="L15" s="177"/>
-    </row>
-    <row r="16" spans="1:14" s="2" customFormat="1" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="26">
+      <c r="L14" s="165"/>
+    </row>
+    <row r="15" spans="1:14" s="2" customFormat="1" ht="15" x14ac:dyDescent="0.25">
+      <c r="A15" s="190"/>
+      <c r="B15" s="191"/>
+      <c r="C15" s="191"/>
+      <c r="D15" s="191"/>
+      <c r="E15" s="191"/>
+      <c r="F15" s="192"/>
+      <c r="G15" s="192"/>
+      <c r="H15" s="191"/>
+      <c r="I15" s="191"/>
+      <c r="J15" s="191"/>
+      <c r="K15" s="192"/>
+      <c r="L15" s="192"/>
+    </row>
+    <row r="16" spans="1:14" s="2" customFormat="1" ht="55.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="201">
+        <v>46030</v>
+      </c>
+      <c r="B16" s="207" t="s">
+        <v>90</v>
+      </c>
+      <c r="C16" s="207"/>
+      <c r="D16" s="207"/>
+      <c r="E16" s="207"/>
+      <c r="F16" s="208" t="s">
+        <v>83</v>
+      </c>
+      <c r="G16" s="208"/>
+      <c r="H16" s="198" t="s">
+        <v>85</v>
+      </c>
+      <c r="I16" s="199"/>
+      <c r="J16" s="200"/>
+      <c r="K16" s="196"/>
+      <c r="L16" s="197"/>
+    </row>
+    <row r="17" spans="1:12" s="2" customFormat="1" ht="47.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="193">
+        <v>46031</v>
+      </c>
+      <c r="B17" s="202" t="s">
+        <v>89</v>
+      </c>
+      <c r="C17" s="202"/>
+      <c r="D17" s="202"/>
+      <c r="E17" s="202"/>
+      <c r="F17" s="208" t="s">
+        <v>83</v>
+      </c>
+      <c r="G17" s="208"/>
+      <c r="H17" s="198" t="s">
+        <v>84</v>
+      </c>
+      <c r="I17" s="199"/>
+      <c r="J17" s="200"/>
+      <c r="K17" s="196"/>
+      <c r="L17" s="197"/>
+    </row>
+    <row r="18" spans="1:12" s="2" customFormat="1" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="193">
         <v>46035</v>
       </c>
-      <c r="B16" s="159" t="s">
+      <c r="B18" s="202" t="s">
+        <v>91</v>
+      </c>
+      <c r="C18" s="202"/>
+      <c r="D18" s="202"/>
+      <c r="E18" s="202"/>
+      <c r="F18" s="209" t="s">
+        <v>71</v>
+      </c>
+      <c r="G18" s="209"/>
+      <c r="H18" s="202" t="s">
         <v>69</v>
       </c>
-      <c r="C16" s="159"/>
-      <c r="D16" s="159"/>
-      <c r="E16" s="159"/>
-      <c r="F16" s="160" t="s">
-        <v>75</v>
-      </c>
-      <c r="G16" s="160"/>
-      <c r="H16" s="159" t="s">
+      <c r="I18" s="202"/>
+      <c r="J18" s="202"/>
+      <c r="K18" s="194"/>
+      <c r="L18" s="195"/>
+    </row>
+    <row r="19" spans="1:12" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="26">
+        <v>46041</v>
+      </c>
+      <c r="B19" s="184" t="s">
+        <v>100</v>
+      </c>
+      <c r="C19" s="184"/>
+      <c r="D19" s="184"/>
+      <c r="E19" s="184"/>
+      <c r="F19" s="185" t="s">
         <v>71</v>
       </c>
-      <c r="I16" s="159"/>
-      <c r="J16" s="159"/>
-      <c r="K16" s="160"/>
-      <c r="L16" s="161"/>
-    </row>
-    <row r="17" spans="1:13" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="26">
-        <v>46041</v>
-      </c>
-      <c r="B17" s="162" t="s">
+      <c r="G19" s="185"/>
+      <c r="H19" s="184" t="s">
         <v>70</v>
       </c>
-      <c r="C17" s="162"/>
-      <c r="D17" s="162"/>
-      <c r="E17" s="162"/>
-      <c r="F17" s="157" t="s">
-        <v>75</v>
-      </c>
-      <c r="G17" s="157"/>
-      <c r="H17" s="162" t="s">
-        <v>72</v>
-      </c>
-      <c r="I17" s="162"/>
-      <c r="J17" s="162"/>
-      <c r="K17" s="157"/>
-      <c r="L17" s="158"/>
-    </row>
-    <row r="18" spans="1:13" s="2" customFormat="1" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="27">
+      <c r="I19" s="184"/>
+      <c r="J19" s="184"/>
+      <c r="K19" s="154"/>
+      <c r="L19" s="158"/>
+    </row>
+    <row r="20" spans="1:12" s="2" customFormat="1" ht="32.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="193">
+        <v>46044</v>
+      </c>
+      <c r="B20" s="203" t="s">
+        <v>99</v>
+      </c>
+      <c r="C20" s="204"/>
+      <c r="D20" s="204"/>
+      <c r="E20" s="205"/>
+      <c r="F20" s="208" t="s">
+        <v>83</v>
+      </c>
+      <c r="G20" s="208"/>
+      <c r="H20" s="218" t="s">
+        <v>104</v>
+      </c>
+      <c r="I20" s="204"/>
+      <c r="J20" s="205"/>
+      <c r="K20" s="206"/>
+      <c r="L20" s="217"/>
+    </row>
+    <row r="21" spans="1:12" s="2" customFormat="1" ht="32.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="193">
+        <v>46051</v>
+      </c>
+      <c r="B21" s="203" t="s">
+        <v>98</v>
+      </c>
+      <c r="C21" s="204"/>
+      <c r="D21" s="204"/>
+      <c r="E21" s="205"/>
+      <c r="F21" s="208" t="s">
+        <v>83</v>
+      </c>
+      <c r="G21" s="208"/>
+      <c r="H21" s="204" t="s">
+        <v>106</v>
+      </c>
+      <c r="I21" s="204"/>
+      <c r="J21" s="205"/>
+      <c r="K21" s="206"/>
+      <c r="L21" s="217"/>
+    </row>
+    <row r="22" spans="1:12" s="2" customFormat="1" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="27">
         <v>46069</v>
       </c>
-      <c r="B18" s="163" t="s">
-        <v>73</v>
-      </c>
-      <c r="C18" s="163"/>
-      <c r="D18" s="163"/>
-      <c r="E18" s="163"/>
-      <c r="F18" s="157" t="s">
-        <v>75</v>
-      </c>
-      <c r="G18" s="157"/>
-      <c r="H18" s="163" t="s">
-        <v>74</v>
-      </c>
-      <c r="I18" s="163"/>
-      <c r="J18" s="163"/>
-      <c r="K18" s="157"/>
-      <c r="L18" s="158"/>
-    </row>
-    <row r="19" spans="1:13" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="27"/>
-      <c r="B19" s="162"/>
-      <c r="C19" s="162"/>
-      <c r="D19" s="162"/>
-      <c r="E19" s="162"/>
-      <c r="F19" s="157"/>
-      <c r="G19" s="157"/>
-      <c r="H19" s="162"/>
-      <c r="I19" s="162"/>
-      <c r="J19" s="162"/>
-      <c r="K19" s="157"/>
-      <c r="L19" s="158"/>
-    </row>
-    <row r="20" spans="1:13" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="27"/>
-      <c r="B20" s="162"/>
-      <c r="C20" s="162"/>
-      <c r="D20" s="162"/>
-      <c r="E20" s="162"/>
-      <c r="F20" s="157"/>
-      <c r="G20" s="157"/>
-      <c r="H20" s="162"/>
-      <c r="I20" s="162"/>
-      <c r="J20" s="162"/>
-      <c r="K20" s="157"/>
-      <c r="L20" s="158"/>
-    </row>
-    <row r="21" spans="1:13" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="27"/>
-      <c r="B21" s="162"/>
-      <c r="C21" s="162"/>
-      <c r="D21" s="162"/>
-      <c r="E21" s="162"/>
-      <c r="F21" s="157"/>
-      <c r="G21" s="157"/>
-      <c r="H21" s="162"/>
-      <c r="I21" s="162"/>
-      <c r="J21" s="162"/>
-      <c r="K21" s="157"/>
-      <c r="L21" s="158"/>
-    </row>
-    <row r="22" spans="1:13" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="27"/>
-      <c r="B22" s="162"/>
-      <c r="C22" s="162"/>
-      <c r="D22" s="162"/>
-      <c r="E22" s="162"/>
-      <c r="F22" s="157"/>
-      <c r="G22" s="157"/>
-      <c r="H22" s="162"/>
-      <c r="I22" s="162"/>
-      <c r="J22" s="162"/>
-      <c r="K22" s="157"/>
-      <c r="L22" s="158"/>
-    </row>
-    <row r="23" spans="1:13" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="27"/>
-      <c r="B23" s="162"/>
-      <c r="C23" s="162"/>
-      <c r="D23" s="162"/>
-      <c r="E23" s="162"/>
-      <c r="F23" s="157"/>
-      <c r="G23" s="157"/>
-      <c r="H23" s="162"/>
-      <c r="I23" s="162"/>
-      <c r="J23" s="162"/>
-      <c r="K23" s="157"/>
-      <c r="L23" s="158"/>
-    </row>
-    <row r="24" spans="1:13" s="2" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="27"/>
-      <c r="B24" s="162"/>
-      <c r="C24" s="162"/>
-      <c r="D24" s="162"/>
-      <c r="E24" s="162"/>
-      <c r="F24" s="157"/>
-      <c r="G24" s="157"/>
-      <c r="H24" s="162"/>
-      <c r="I24" s="162"/>
-      <c r="J24" s="162"/>
-      <c r="K24" s="157"/>
+      <c r="B22" s="203" t="s">
+        <v>87</v>
+      </c>
+      <c r="C22" s="204"/>
+      <c r="D22" s="204"/>
+      <c r="E22" s="205"/>
+      <c r="F22" s="186" t="s">
+        <v>71</v>
+      </c>
+      <c r="G22" s="187"/>
+      <c r="H22" s="203" t="s">
+        <v>86</v>
+      </c>
+      <c r="I22" s="204"/>
+      <c r="J22" s="205"/>
+      <c r="K22" s="188"/>
+      <c r="L22" s="189"/>
+    </row>
+    <row r="23" spans="1:12" s="2" customFormat="1" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="27">
+        <v>46072</v>
+      </c>
+      <c r="B23" s="203" t="s">
+        <v>107</v>
+      </c>
+      <c r="C23" s="204"/>
+      <c r="D23" s="204"/>
+      <c r="E23" s="205"/>
+      <c r="F23" s="208" t="s">
+        <v>83</v>
+      </c>
+      <c r="G23" s="208"/>
+      <c r="H23" s="203" t="s">
+        <v>108</v>
+      </c>
+      <c r="I23" s="204"/>
+      <c r="J23" s="205"/>
+      <c r="K23" s="206"/>
+      <c r="L23" s="217"/>
+    </row>
+    <row r="24" spans="1:12" s="2" customFormat="1" ht="39" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="27">
+        <v>46083</v>
+      </c>
+      <c r="B24" s="184" t="s">
+        <v>94</v>
+      </c>
+      <c r="C24" s="184"/>
+      <c r="D24" s="184"/>
+      <c r="E24" s="184"/>
+      <c r="F24" s="186" t="s">
+        <v>71</v>
+      </c>
+      <c r="G24" s="187"/>
+      <c r="H24" s="184" t="s">
+        <v>95</v>
+      </c>
+      <c r="I24" s="184"/>
+      <c r="J24" s="184"/>
+      <c r="K24" s="154"/>
       <c r="L24" s="158"/>
     </row>
-    <row r="25" spans="1:13" s="2" customFormat="1" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="28"/>
-      <c r="B25" s="164"/>
-      <c r="C25" s="164"/>
-      <c r="D25" s="164"/>
-      <c r="E25" s="164"/>
-      <c r="F25" s="190"/>
-      <c r="G25" s="190"/>
-      <c r="H25" s="164"/>
-      <c r="I25" s="164"/>
-      <c r="J25" s="164"/>
-      <c r="K25" s="190"/>
-      <c r="L25" s="191"/>
-    </row>
-    <row r="26" spans="1:13" s="2" customFormat="1" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="3"/>
-      <c r="B26" s="3"/>
-      <c r="C26" s="4" t="s">
+    <row r="25" spans="1:12" s="2" customFormat="1" ht="39" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="27">
+        <v>46086</v>
+      </c>
+      <c r="B25" s="203" t="s">
+        <v>109</v>
+      </c>
+      <c r="C25" s="204"/>
+      <c r="D25" s="204"/>
+      <c r="E25" s="219"/>
+      <c r="F25" s="208" t="s">
+        <v>83</v>
+      </c>
+      <c r="G25" s="208"/>
+      <c r="H25" s="218" t="s">
+        <v>110</v>
+      </c>
+      <c r="I25" s="204"/>
+      <c r="J25" s="205"/>
+      <c r="K25" s="206"/>
+      <c r="L25" s="217"/>
+    </row>
+    <row r="26" spans="1:12" s="2" customFormat="1" ht="54" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="27">
+        <v>46093</v>
+      </c>
+      <c r="B26" s="203" t="s">
+        <v>111</v>
+      </c>
+      <c r="C26" s="204"/>
+      <c r="D26" s="204"/>
+      <c r="E26" s="204"/>
+      <c r="F26" s="208" t="s">
+        <v>83</v>
+      </c>
+      <c r="G26" s="208"/>
+      <c r="H26" s="204" t="s">
+        <v>112</v>
+      </c>
+      <c r="I26" s="204"/>
+      <c r="J26" s="205"/>
+      <c r="K26" s="206"/>
+      <c r="L26" s="217"/>
+    </row>
+    <row r="27" spans="1:12" s="2" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="27">
+        <v>46094</v>
+      </c>
+      <c r="B27" s="203" t="s">
+        <v>88</v>
+      </c>
+      <c r="C27" s="204"/>
+      <c r="D27" s="204"/>
+      <c r="E27" s="205"/>
+      <c r="F27" s="186" t="s">
+        <v>71</v>
+      </c>
+      <c r="G27" s="187"/>
+      <c r="H27" s="203" t="s">
+        <v>92</v>
+      </c>
+      <c r="I27" s="204"/>
+      <c r="J27" s="205"/>
+      <c r="K27" s="188"/>
+      <c r="L27" s="189"/>
+    </row>
+    <row r="28" spans="1:12" s="2" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="27">
+        <v>46100</v>
+      </c>
+      <c r="B28" s="203" t="s">
+        <v>114</v>
+      </c>
+      <c r="C28" s="204"/>
+      <c r="D28" s="204"/>
+      <c r="E28" s="205"/>
+      <c r="F28" s="208" t="s">
+        <v>83</v>
+      </c>
+      <c r="G28" s="208"/>
+      <c r="H28" s="203" t="s">
+        <v>113</v>
+      </c>
+      <c r="I28" s="204"/>
+      <c r="J28" s="205"/>
+      <c r="K28" s="206"/>
+      <c r="L28" s="217"/>
+    </row>
+    <row r="29" spans="1:12" s="2" customFormat="1" ht="49.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="27">
+        <v>46106</v>
+      </c>
+      <c r="B29" s="184" t="s">
+        <v>103</v>
+      </c>
+      <c r="C29" s="184"/>
+      <c r="D29" s="184"/>
+      <c r="E29" s="184"/>
+      <c r="F29" s="185" t="s">
+        <v>71</v>
+      </c>
+      <c r="G29" s="185"/>
+      <c r="H29" s="184" t="s">
+        <v>105</v>
+      </c>
+      <c r="I29" s="184"/>
+      <c r="J29" s="184"/>
+      <c r="K29" s="154"/>
+      <c r="L29" s="158"/>
+    </row>
+    <row r="30" spans="1:12" s="2" customFormat="1" ht="49.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="27">
+        <v>46107</v>
+      </c>
+      <c r="B30" s="203" t="s">
+        <v>115</v>
+      </c>
+      <c r="C30" s="204"/>
+      <c r="D30" s="204"/>
+      <c r="E30" s="205"/>
+      <c r="F30" s="208" t="s">
+        <v>83</v>
+      </c>
+      <c r="G30" s="208"/>
+      <c r="H30" s="203" t="s">
+        <v>116</v>
+      </c>
+      <c r="I30" s="204"/>
+      <c r="J30" s="205"/>
+      <c r="K30" s="188"/>
+      <c r="L30" s="189"/>
+    </row>
+    <row r="31" spans="1:12" s="2" customFormat="1" ht="49.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="27">
+        <v>46112</v>
+      </c>
+      <c r="B31" s="203" t="s">
+        <v>117</v>
+      </c>
+      <c r="C31" s="204"/>
+      <c r="D31" s="204"/>
+      <c r="E31" s="205"/>
+      <c r="F31" s="208" t="s">
+        <v>83</v>
+      </c>
+      <c r="G31" s="208"/>
+      <c r="H31" s="203" t="s">
+        <v>118</v>
+      </c>
+      <c r="I31" s="204"/>
+      <c r="J31" s="205"/>
+      <c r="K31" s="206"/>
+      <c r="L31" s="217"/>
+    </row>
+    <row r="32" spans="1:12" s="2" customFormat="1" ht="69" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="27">
+        <v>46115</v>
+      </c>
+      <c r="B32" s="203" t="s">
+        <v>119</v>
+      </c>
+      <c r="C32" s="204"/>
+      <c r="D32" s="204"/>
+      <c r="E32" s="205"/>
+      <c r="F32" s="208" t="s">
+        <v>83</v>
+      </c>
+      <c r="G32" s="208"/>
+      <c r="H32" s="218" t="s">
+        <v>120</v>
+      </c>
+      <c r="I32" s="204"/>
+      <c r="J32" s="205"/>
+      <c r="K32" s="206"/>
+      <c r="L32" s="217"/>
+    </row>
+    <row r="33" spans="1:13" s="2" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="27">
+        <v>46118</v>
+      </c>
+      <c r="B33" s="184" t="s">
+        <v>102</v>
+      </c>
+      <c r="C33" s="184"/>
+      <c r="D33" s="184"/>
+      <c r="E33" s="184"/>
+      <c r="F33" s="185" t="s">
+        <v>93</v>
+      </c>
+      <c r="G33" s="185"/>
+      <c r="H33" s="210" t="s">
+        <v>96</v>
+      </c>
+      <c r="I33" s="211"/>
+      <c r="J33" s="212"/>
+      <c r="K33" s="154"/>
+      <c r="L33" s="158"/>
+    </row>
+    <row r="34" spans="1:13" s="2" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="27">
+        <v>46118</v>
+      </c>
+      <c r="B34" s="184" t="s">
+        <v>102</v>
+      </c>
+      <c r="C34" s="184"/>
+      <c r="D34" s="184"/>
+      <c r="E34" s="184"/>
+      <c r="F34" s="185" t="s">
+        <v>71</v>
+      </c>
+      <c r="G34" s="185"/>
+      <c r="H34" s="213"/>
+      <c r="I34" s="214"/>
+      <c r="J34" s="215"/>
+      <c r="K34" s="154"/>
+      <c r="L34" s="158"/>
+    </row>
+    <row r="35" spans="1:13" s="2" customFormat="1" ht="42.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="28">
+        <v>46121</v>
+      </c>
+      <c r="B35" s="157" t="s">
+        <v>101</v>
+      </c>
+      <c r="C35" s="157"/>
+      <c r="D35" s="157"/>
+      <c r="E35" s="157"/>
+      <c r="F35" s="185" t="s">
+        <v>93</v>
+      </c>
+      <c r="G35" s="185"/>
+      <c r="H35" s="216" t="s">
+        <v>97</v>
+      </c>
+      <c r="I35" s="216"/>
+      <c r="J35" s="216"/>
+      <c r="K35" s="155"/>
+      <c r="L35" s="160"/>
+    </row>
+    <row r="36" spans="1:13" s="2" customFormat="1" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="3"/>
+      <c r="B36" s="3"/>
+      <c r="C36" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="D26" s="4"/>
-      <c r="E26" s="4" t="s">
+      <c r="D36" s="4"/>
+      <c r="E36" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="G26" s="4" t="s">
+      <c r="G36" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="H26" s="4"/>
-      <c r="J26" s="4" t="s">
+      <c r="H36" s="4"/>
+      <c r="J36" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="K26" s="4"/>
-      <c r="L26" s="3"/>
-    </row>
-    <row r="27" spans="1:13" s="2" customFormat="1" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="3"/>
-      <c r="B27" s="3"/>
-      <c r="C27" s="4"/>
-      <c r="D27" s="4"/>
-      <c r="E27" s="4" t="s">
+      <c r="K36" s="4"/>
+      <c r="L36" s="3"/>
+    </row>
+    <row r="37" spans="1:13" s="2" customFormat="1" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="3"/>
+      <c r="B37" s="3"/>
+      <c r="C37" s="4"/>
+      <c r="D37" s="4"/>
+      <c r="E37" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="G27" s="4" t="s">
+      <c r="G37" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="H27" s="4"/>
-      <c r="J27" s="4"/>
-      <c r="K27" s="4"/>
-      <c r="L27" s="3"/>
-    </row>
-    <row r="28" spans="1:13" s="2" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="3"/>
-      <c r="B28" s="3"/>
-      <c r="C28" s="4"/>
-      <c r="D28" s="4"/>
-      <c r="E28" s="4"/>
-      <c r="G28" s="4"/>
-      <c r="H28" s="4"/>
-      <c r="J28" s="4"/>
-      <c r="K28" s="4"/>
-      <c r="L28" s="3"/>
-    </row>
-    <row r="29" spans="1:13" s="2" customFormat="1" ht="29.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B29" s="193" t="str">
+      <c r="H37" s="4"/>
+      <c r="J37" s="4"/>
+      <c r="K37" s="4"/>
+      <c r="L37" s="3"/>
+    </row>
+    <row r="38" spans="1:13" s="2" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="3"/>
+      <c r="B38" s="3"/>
+      <c r="C38" s="4"/>
+      <c r="D38" s="4"/>
+      <c r="E38" s="4"/>
+      <c r="G38" s="4"/>
+      <c r="H38" s="4"/>
+      <c r="J38" s="4"/>
+      <c r="K38" s="4"/>
+      <c r="L38" s="3"/>
+    </row>
+    <row r="39" spans="1:13" s="2" customFormat="1" ht="29.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B39" s="156" t="str">
         <f>'Asignación de Proyecto'!J34</f>
         <v>M. C. Nélida Báron Pérez</v>
       </c>
-      <c r="C29" s="193"/>
-      <c r="D29" s="193"/>
-      <c r="E29" s="193"/>
-      <c r="H29" s="189"/>
-      <c r="I29" s="189"/>
-      <c r="J29" s="189"/>
-      <c r="K29" s="189"/>
-    </row>
-    <row r="30" spans="1:13" s="2" customFormat="1" ht="15.6" x14ac:dyDescent="0.25">
-      <c r="B30" s="192" t="str">
+      <c r="C39" s="156"/>
+      <c r="D39" s="156"/>
+      <c r="E39" s="156"/>
+      <c r="H39" s="159"/>
+      <c r="I39" s="159"/>
+      <c r="J39" s="159"/>
+      <c r="K39" s="159"/>
+    </row>
+    <row r="40" spans="1:13" s="2" customFormat="1" ht="15.6" x14ac:dyDescent="0.25">
+      <c r="B40" s="153" t="str">
         <f>'Asignación de Proyecto'!J35</f>
         <v>ASESORA UNIVERSITARIA</v>
       </c>
-      <c r="C30" s="192"/>
-      <c r="D30" s="192"/>
-      <c r="E30" s="192"/>
-      <c r="H30" s="192" t="s">
-        <v>51</v>
-      </c>
-      <c r="I30" s="192"/>
-      <c r="J30" s="192"/>
-      <c r="K30" s="192"/>
-    </row>
-    <row r="31" spans="1:13" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="83" t="s">
+      <c r="C40" s="153"/>
+      <c r="D40" s="153"/>
+      <c r="E40" s="153"/>
+      <c r="H40" s="153" t="s">
+        <v>53</v>
+      </c>
+      <c r="I40" s="153"/>
+      <c r="J40" s="153"/>
+      <c r="K40" s="153"/>
+    </row>
+    <row r="41" spans="1:13" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="108" t="s">
         <v>47</v>
       </c>
-      <c r="B31" s="83"/>
-      <c r="C31" s="83"/>
-      <c r="D31" s="83"/>
-      <c r="E31" s="83"/>
-      <c r="F31" s="83"/>
-      <c r="G31" s="83"/>
-      <c r="H31" s="83"/>
-      <c r="I31" s="83"/>
-      <c r="J31" s="83"/>
-      <c r="K31" s="83"/>
-      <c r="L31" s="83"/>
-      <c r="M31" s="18"/>
-    </row>
-    <row r="32" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="33" ht="63.9" customHeight="1" x14ac:dyDescent="0.25"/>
+      <c r="B41" s="108"/>
+      <c r="C41" s="108"/>
+      <c r="D41" s="108"/>
+      <c r="E41" s="108"/>
+      <c r="F41" s="108"/>
+      <c r="G41" s="108"/>
+      <c r="H41" s="108"/>
+      <c r="I41" s="108"/>
+      <c r="J41" s="108"/>
+      <c r="K41" s="108"/>
+      <c r="L41" s="108"/>
+      <c r="M41" s="18"/>
+    </row>
+    <row r="42" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="43" spans="1:13" ht="63.9" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <mergeCells count="67">
+  <mergeCells count="98">
+    <mergeCell ref="B28:E28"/>
+    <mergeCell ref="F28:G28"/>
+    <mergeCell ref="H28:J28"/>
     <mergeCell ref="B30:E30"/>
-    <mergeCell ref="H30:K30"/>
-    <mergeCell ref="F22:G22"/>
-    <mergeCell ref="F23:G23"/>
-    <mergeCell ref="F24:G24"/>
-    <mergeCell ref="F25:G25"/>
-    <mergeCell ref="B29:E29"/>
-    <mergeCell ref="H22:J22"/>
-    <mergeCell ref="H23:J23"/>
-    <mergeCell ref="H24:J24"/>
+    <mergeCell ref="F30:G30"/>
+    <mergeCell ref="H30:J30"/>
+    <mergeCell ref="B25:E25"/>
     <mergeCell ref="H25:J25"/>
-    <mergeCell ref="K22:L22"/>
-    <mergeCell ref="K23:L23"/>
-    <mergeCell ref="K24:L24"/>
+    <mergeCell ref="B26:E26"/>
+    <mergeCell ref="F26:G26"/>
+    <mergeCell ref="H26:J26"/>
+    <mergeCell ref="K17:L17"/>
+    <mergeCell ref="B27:E27"/>
+    <mergeCell ref="H27:J27"/>
+    <mergeCell ref="K27:L27"/>
+    <mergeCell ref="F27:G27"/>
+    <mergeCell ref="B20:E20"/>
     <mergeCell ref="F20:G20"/>
     <mergeCell ref="H20:J20"/>
+    <mergeCell ref="B21:E21"/>
+    <mergeCell ref="F21:G21"/>
     <mergeCell ref="H21:J21"/>
-    <mergeCell ref="H29:K29"/>
-    <mergeCell ref="K25:L25"/>
-    <mergeCell ref="K20:L20"/>
-    <mergeCell ref="K21:L21"/>
+    <mergeCell ref="B23:E23"/>
+    <mergeCell ref="H23:J23"/>
+    <mergeCell ref="F23:G23"/>
+    <mergeCell ref="A14:A15"/>
+    <mergeCell ref="F19:G19"/>
+    <mergeCell ref="B18:E18"/>
+    <mergeCell ref="F18:G18"/>
+    <mergeCell ref="H18:J18"/>
+    <mergeCell ref="K18:L18"/>
+    <mergeCell ref="B16:E16"/>
+    <mergeCell ref="B17:E17"/>
+    <mergeCell ref="F16:G16"/>
+    <mergeCell ref="F17:G17"/>
+    <mergeCell ref="H16:J16"/>
+    <mergeCell ref="H17:J17"/>
+    <mergeCell ref="K16:L16"/>
+    <mergeCell ref="A41:L41"/>
+    <mergeCell ref="B19:E19"/>
+    <mergeCell ref="B22:E22"/>
+    <mergeCell ref="B24:E24"/>
+    <mergeCell ref="B29:E29"/>
+    <mergeCell ref="B33:E33"/>
+    <mergeCell ref="B34:E34"/>
+    <mergeCell ref="B35:E35"/>
+    <mergeCell ref="H19:J19"/>
+    <mergeCell ref="F24:G24"/>
+    <mergeCell ref="K19:L19"/>
+    <mergeCell ref="A2:J2"/>
+    <mergeCell ref="A3:J3"/>
+    <mergeCell ref="A4:J4"/>
+    <mergeCell ref="C5:L5"/>
+    <mergeCell ref="K6:L6"/>
     <mergeCell ref="K8:L8"/>
     <mergeCell ref="C9:L9"/>
     <mergeCell ref="K7:L7"/>
@@ -3672,45 +4284,43 @@
     <mergeCell ref="A11:B11"/>
     <mergeCell ref="A12:B12"/>
     <mergeCell ref="A13:B13"/>
-    <mergeCell ref="A2:J2"/>
-    <mergeCell ref="A3:J3"/>
-    <mergeCell ref="A4:J4"/>
-    <mergeCell ref="C5:L5"/>
-    <mergeCell ref="K6:L6"/>
-    <mergeCell ref="A31:L31"/>
-    <mergeCell ref="B17:E17"/>
-    <mergeCell ref="B18:E18"/>
-    <mergeCell ref="B19:E19"/>
-    <mergeCell ref="B20:E20"/>
-    <mergeCell ref="B21:E21"/>
-    <mergeCell ref="B22:E22"/>
-    <mergeCell ref="B23:E23"/>
-    <mergeCell ref="B24:E24"/>
-    <mergeCell ref="B25:E25"/>
-    <mergeCell ref="H17:J17"/>
-    <mergeCell ref="H18:J18"/>
-    <mergeCell ref="H19:J19"/>
-    <mergeCell ref="F21:G21"/>
-    <mergeCell ref="K17:L17"/>
-    <mergeCell ref="K18:L18"/>
-    <mergeCell ref="A14:A15"/>
-    <mergeCell ref="F19:G19"/>
-    <mergeCell ref="K19:L19"/>
-    <mergeCell ref="F17:G17"/>
-    <mergeCell ref="F18:G18"/>
-    <mergeCell ref="B16:E16"/>
-    <mergeCell ref="F16:G16"/>
-    <mergeCell ref="H16:J16"/>
-    <mergeCell ref="K16:L16"/>
+    <mergeCell ref="F22:G22"/>
+    <mergeCell ref="H22:J22"/>
+    <mergeCell ref="H24:J24"/>
+    <mergeCell ref="H39:K39"/>
+    <mergeCell ref="K35:L35"/>
+    <mergeCell ref="K22:L22"/>
+    <mergeCell ref="K24:L24"/>
+    <mergeCell ref="H33:J34"/>
+    <mergeCell ref="F25:G25"/>
+    <mergeCell ref="K30:L30"/>
+    <mergeCell ref="F31:G31"/>
+    <mergeCell ref="H31:J31"/>
+    <mergeCell ref="F32:G32"/>
+    <mergeCell ref="H32:J32"/>
+    <mergeCell ref="B40:E40"/>
+    <mergeCell ref="H40:K40"/>
+    <mergeCell ref="F29:G29"/>
+    <mergeCell ref="F33:G33"/>
+    <mergeCell ref="F34:G34"/>
+    <mergeCell ref="F35:G35"/>
+    <mergeCell ref="B39:E39"/>
+    <mergeCell ref="H29:J29"/>
+    <mergeCell ref="H35:J35"/>
+    <mergeCell ref="K29:L29"/>
+    <mergeCell ref="K33:L33"/>
+    <mergeCell ref="K34:L34"/>
+    <mergeCell ref="B31:E31"/>
+    <mergeCell ref="B32:E32"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Selecciona directora o director." prompt="Selecciona directora o director." sqref="H30:K30" xr:uid="{00000000-0002-0000-0100-000000000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Selecciona directora o director." prompt="Selecciona directora o director." sqref="H40:K40" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>$N$5:$N$7</formula1>
     </dataValidation>
   </dataValidations>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.19685039370078741" right="0.19685039370078741" top="0.39370078740157483" bottom="0.39370078740157483" header="0" footer="0"/>
-  <pageSetup scale="79" orientation="landscape" r:id="rId1"/>
+  <pageSetup scale="60" orientation="portrait" r:id="rId1"/>
   <headerFooter alignWithMargins="0"/>
   <drawing r:id="rId2"/>
 </worksheet>

</xml_diff>